<commit_message>
Implement Destiny Matrix compatibility support: dual inputs, compatibility sheet sync, tab filters, program highlights, and Script Board real-time synchronization
</commit_message>
<xml_diff>
--- a/data/interpretations.xlsx
+++ b/data/interpretations.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master_Database" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compatibility" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -14872,4 +14873,122 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Position Meaning</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Interpretation Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Combined Portrait</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>General Compatibility</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Combined Portrait Number 3 reading text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Combined Core</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Love Dynamics</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Combined Core Number 10 Love Alignment reading text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>M-N-D</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Compatibility Program</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Compatibility Program</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>15-20-5</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Rebel Compatibility Program (15-20-5) reading text.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement yearly and couple forecast engine with interactive UI, data synchronization, and age-based calculation logic
</commit_message>
<xml_diff>
--- a/data/interpretations.xlsx
+++ b/data/interpretations.xlsx
@@ -309,7 +309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E618"/>
+  <dimension ref="A1:E664"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="7" min="1" max="1"/>
@@ -14870,6 +14870,1303 @@
         </is>
       </c>
     </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>1</v>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>The Magician. The Pioneer.** 
+_Only in the personal forecast — in the year of birth and at ages 20, 40, 60 (at 40 and 60 as the second energy)._ 
+This is one of the most powerful periods in a person’s life. Everything you conceive has a chance to take form. Ideas find shape, plans come to life, doors open where before there was a dead end. This is a time of active movement forward. New knowledge, new contacts, new projects. The mind is literally tuned to absorb information — learn, soak it up, grow. Promotions, business launches, creative breakthroughs are all possible. 
+You are seen. You are heard. In this period you are able to inspire others — simply by your presence and your word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>What to watch for</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>1</v>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>The main trap of this period is overconfidence. A sense of superiority can turn into conflicts and a loss of authority. Watch your documents — mistakes and misunderstandings are possible. Control your thoughts — in this period they materialize with doubled force.</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>1</v>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>Set goals and write them down. Seek collaboration with professionals. Strengthen the body — especially the spine and the lower part. Practice meditation. Visit places of power. And work on your self-worth — this period manifests exactly as much as you believe in yourself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>2</v>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>The High Priestess. Unity and Harmony.** 
+### _In the personal forecast — in the year of birth, and at ages 10, 20, 40, and 60. In a couple’s forecast it appears extremely rarely._ 
+This is a period of silence and depth. A time when there’s no need to storm and conquer — there’s a need to listen. Listen to yourself, listen to life, trust what is happening. 
+Intuition sharpens to its limit in this period. Information that was long hidden may open to you. Secrets surface, the concealed comes to light. Don’t ask — just observe. The answers will come on their own. 
+This is a soft, spiritual period. A good time for learning, gathering information, developing inner abilities. Relationships with the mother and the women of the lineage come to the foreground — it’s important to harmonize them. Joyful events connected with children are possible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>What to watch for</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>2</v>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>The main trap is trying to control everything with logic. It doesn’t work here. Also dangerous are intrigues, gossip, participation in others’ games. A third party may appear in the relationship — a woman who brings instability. Watch the information you pass on and receive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>2</v>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>Trust your intuition — in this period it is your main instrument. Record important promises in writing. Practice yoga, meditation, pranayama. Create a harmonious space around you. Watch your nutrition — more natural and plant-based. And remember — the world is not divided into black and white.</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>3</v>
+      </c>
+      <c r="E625" t="inlineStr">
+        <is>
+          <t>The Empress. Fertility and Femininity.** 
+### _One of the richest periods — both for the personal forecast and for the couple._ **Personal forecast** 
+This is a time when feminine energy comes to the foreground — in both partners, regardless of gender. Emotionality, intuition, creativity, beauty, the desire to surround yourself with comfort and fullness — all of this blossoms in this period. 
+The material sphere strengthens. Income, real estate purchases, career advancements are possible. Creative ideas come to life easily. The period is favorable for relationships — a romantic, courtship stage, conversations about continuing the family, attention from the opposite sex. **For a woman** — this is the peak of femininity and desirability, a chance to marry, become a mother, gain a home and status. 
+**For a man** — a period when he naturally takes on the role of provider and is surrounded by women’s attention. 
+The main trap is the loss of balance. A woman may slip into aggression and control, taking on masculine roles. A man may lose his masculinity, or on the contrary, slip into idleness. It’s important to stay in your own nature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>3</v>
+      </c>
+      <c r="E626" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+For women — manicures, spa, jewelry, time with friends, get-togethers, repairing broken jewelry. Mend the relationship with your mother. Delegate domestic tasks. For men — do something kind for the women of the lineage, voice your boundaries to your partner, take responsibility.</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>4</v>
+      </c>
+      <c r="E627" t="inlineStr">
+        <is>
+          <t>The Emperor. Power and Responsibility.** 
+### **Personal forecast** 
+This is a powerful period of masculine energy — in both partners regardless of gender. Persistence, decisiveness, organization, logic, active action. A period when you can and should take on responsibility — and get results for it. 
+Career advancements, opening a business, promotions, new positions — all of this becomes real precisely now. Government matters and documents are resolved successfully. Rewards arrive for past investments. 
+**For a man** — one of the best periods for strengthening himself as a leader, provider, father. A very money-rich energy. It’s important not to miss the moment and to act. 
+**For a woman** — a fateful meeting with a man or the patronage of an influential man is possible. But it’s important to make sure you don’t slip into masculine roles — otherwise the energy will start to press on the relationship. 
+The main trap for a woman is taking on too many masculine duties and crushing her partner with authority. The main trap for a man is slipping into rebellion or passivity when responsibility is needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>4</v>
+      </c>
+      <c r="E628" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+**For women** — be softer, accept the man, learn to ask rather than do it all yourself. Work through the relationship with the father. Wear feminine clothing. 
+**For men** — take responsibility consciously, set goals in writing, give time to family and not only to career. Work through the relationship with the mother. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>5</v>
+      </c>
+      <c r="E629" t="inlineStr">
+        <is>
+          <t>The Hierophant. Student and Teacher. Family.** 
+### **Personal forecast** 
+This is a period when family, traditions, and the transmission of knowledge come to the foreground. Everything connected with the lineage, with roots, with relationships between generations — becomes especially important. 
+The period is favorable for learning and spiritual growth. A mentor may appear on your path — someone ready to pass on knowledge and experience. Or, on the contrary — you yourself become a teacher for someone. In this period it’s important not only to accumulate knowledge but to pass it on. 
+Official matters are resolved successfully. A good time for processing documents, entering into marriage, legal questions. Career advancement is possible through authority and the respect of those around you. 
+The main trap is living someone else’s life instead of your own. Clinging too much to relatives, putting yourself in the victim position, lecturing those who didn’t ask. Also dangerous are false teachers and spiritual intoxication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>5</v>
+      </c>
+      <c r="E630" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Put things in order — literally and figuratively. Systematize documents, keep a routine, respect others’ time. Create family traditions. Accept your father — this is the key work of the period. Learn — and immediately pass the knowledge on. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>6</v>
+      </c>
+      <c r="E631" t="inlineStr">
+        <is>
+          <t>The Lovers. Relationships, Choice, and Unconditional Love.** 
+### **Personal forecast** 
+One of the most beautiful and vivid periods in life. Much celebration, laughter, heartfelt conversations, pleasant meetings. Everything connected with beauty, love, and harmony — blossoms. 
+This is a time of new relationships — not only romantic but also business. For those already in a couple — a wonderful moment for deepening closeness or planning a child. The single may meet a great love. 
+A period of right choice — but precisely from the heart, not from the head. Work that isn’t to your liking will drain you. Only what you love — will give results. Communications blossom. Much interaction, new contacts, friends. Hobbies may grow into a profession. Creative projects launch easily and joyfully. The main trap is living by someone else’s script, pleasing everyone, losing yourself. Also dangerous are betrayals, love triangles, betrayals by friends. All of this is given to teach you to distinguish the real from the unreal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>6</v>
+      </c>
+      <c r="E632" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Speak of love — aloud, to loved ones and to yourself. Tend to your appearance and body. Give gifts without expectations. Open the heart through metta meditation. When choosing — listen to the body, not logic. Watch your heart — in the literal sense. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>7</v>
+      </c>
+      <c r="E633" t="inlineStr">
+        <is>
+          <t>The Chariot. Movement and Victory.** 
+### **Personal forecast** 
+This is a period of true breakthrough. A time when you’re like a tank — decisive, driving, seeing no obstacles. Everything that once seemed impossible — becomes achievable precisely now. Career victories, opening a business, launching projects, promotions — all of this is supported by the energy of the period. Travel, relocations, getting a license, sports are favorable. The energy of a winner accompanies you. 
+In relationships — an active sexual life, marriage is possible. 
+The main trap is walking over others, ignoring people in the pursuit of a goal. Or on the contrary — falling into passivity and missing the powerful potential of the period. A lack of movement in this period literally strikes at health and finances.</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>7</v>
+      </c>
+      <c r="E634" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Set goals in writing and break them into small steps. Do sports — it transforms aggression into creation. Rejoice in every victory — big and small. Work with your combativeness — don’t press it onto others, channel it into action. The faster you move — the faster the answers come. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>8</v>
+      </c>
+      <c r="E635" t="inlineStr">
+        <is>
+          <t>Justice. Fairness and Balance.** 
+### **Personal forecast** 
+This is a period of cause and effect. What you sowed before — you reap now. If you acted honestly and wisely — a karmic reward arrives. If not — the bill comes due. 
+A period of balance in everything — work and rest, labor and recovery, giving and receiving. A time of logic and reason rather than emotions. A good moment for rethinking — to stop, look at where you came from and where you’re going. 
+The legal sphere is especially active. Documents, contracts, real estate deals, the official registration of marriage — all of this goes through successfully if you act honestly. Court cases, interaction with state structures — are also characteristic of this period. 
+The main trap is waging war for justice. Fighting against injustice, going to court, accusing. It is precisely this that leads to the minus. Also dangerous are imbalance, burnout, deception, and breaking promises.</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>8</v>
+      </c>
+      <c r="E636" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Maintain balance in all spheres of life — use the wheel of life balance. Be punctual. Don’t take loans and don’t lend money. Control expenses. Keep promises — even those made to yourself. Take the position of an observer rather than a judge. Sow good freely — it will return. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>9</v>
+      </c>
+      <c r="E637" t="inlineStr">
+        <is>
+          <t>The Hermit. Wisdom and the Inner Path.** 
+### **Personal forecast** 
+This is a quiet period. Without sharp swings, without storming and conquering. A time when life invites you inward — to yourself, to your thoughts, to your depth. 
+Spiritual discoveries, creative unfolding, the search for like-minded people and mentors — all of this is characteristic of the nine. A good time for learning, retreats, work with a psychologist or coach. For women the period may mean pregnancy. 
+The desire to be alone — is normal and necessary. This is not depression, it is replenishment. It’s only important to return from solitude in time and not lose connection with loved ones. The main trap is slipping into pride, judging others, closing off from people entirely. Or on the contrary — fearing solitude and not giving yourself the silence you need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>9</v>
+      </c>
+      <c r="E638" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Spend time in nature — it is the best medicine of the period. Shift from the head into the body — bodily practices, massage, floating. Share wisdom through experience rather than through preaching. Listen to insights — they don’t come by chance. Practice grounding. Speak of feelings aloud through “I” statements. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>10</v>
+      </c>
+      <c r="E639" t="inlineStr">
+        <is>
+          <t>The Wheel of Fortune. Flow and Luck.** 
+### **Personal forecast** 
+One of the luckiest periods. Fortune turns its face toward you — and if you are relaxed and open, life itself carries you in the right direction. There’s no need to force and push — there’s a need to trust. 
+Unexpected winnings, large profit, the right people who appear at the right moment, doors that open on their own — all of this is real in the period of the ten. This is a karmic reward for past efforts. A kind of vacation for the soul. 
+Fateful turns and important events — are characteristic of this period. Life changes rapidly. The main thing — not to cling to the old and not to miss new chances. 
+In the sphere of love — both serious meetings and light infatuations are possible. 
+The main trap is passivity and the inability to see signs. Luck comes — but if you don’t notice it and don’t act, it goes to another. It’s also dangerous to fall into a negative flow through your surroundings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>10</v>
+      </c>
+      <c r="E640" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Practice gratitude daily — aloud, in writing, or to yourself. Be grateful for everything including failures. Learn to listen to the body when choosing. Choose positive people around you. Be attentive to signs and opportunities — they flash by quickly. Tell yourself: what’s mine will be mine. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>11</v>
+      </c>
+      <c r="E641" t="inlineStr">
+        <is>
+          <t>Strength and Potential.** 
+### **Personal forecast** 
+This is one of the most powerful periods. A double energy — as if a second wind opens. Everything you planned, dreamed of, postponed — now comes to life. A period for active action; passivity here literally costs dearly. 
+Career successes, the launch of major projects, the creation of organizations and movements — all of this is possible. Physical endurance is at its peak. An excellent period for sports, for challenging yourself, for changing habits and developing willpower. 
+A period of trials — of strength, of passion, of the ability to overcome. But you have everything you need to cope and emerge victorious. 
+Sexual activity is high. Pregnancy is possible — double strength literally means two people. The main trap is suppressing others with an excess of energy, slipping into aggression, working yourself to exhaustion. If the energy isn’t released — it stagnates and strikes at health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>11</v>
+      </c>
+      <c r="E642" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Sports are mandatory — especially in the second half of the day. Alternate activity and rest — like in a workout: tense, relax. Control aggression and the volume of your voice. Set long-term goals and praise yourself for every item crossed off. For women — develop femininity rather than stopping a galloping horse. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>12</v>
+      </c>
+      <c r="E643" t="inlineStr">
+        <is>
+          <t>The Hanged Man. Service and a Different Vision.** 
+### **Personal forecast** 
+Life may turn 180 degrees — literally like the person on the card. And if you look at this not with panic but with interest — you can see what was previously invisible. New solutions, new angles of view, unexpected ways out of long-standing dead ends. 
+This is a period of a different vision. Slow, at times requiring waiting and patience. Something may leave — but in the freed space, something better will surely come. The task is to see new possibilities in what seems like a loss. 
+The desire to serve others, take part in charity, be useful — is characteristic of this period. The main thing is to distinguish service from love and servility from fear or pressure. 
+The period is filled with creativity — any creative projects, courses, practices receive support. The main trap is slipping into victimhood. Doing something against yourself, allowing yourself to be used, rescuing those who didn’t ask. Also dangerous are indecision and fear of change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>12</v>
+      </c>
+      <c r="E644" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Don’t sacrifice yourself — neither in work nor in relationships. Learn to say no. Before helping — ask whether help is needed. Give yourself gifts and praise yourself. Accept compliments without deflecting. Engage in creativity. Help from fullness rather than from your last reserves. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>13</v>
+      </c>
+      <c r="E645" t="inlineStr">
+        <is>
+          <t>Death. Transformation and Rebirth.** 
+### **Personal forecast** 
+This is one of the most powerful periods of transformation. Life may divide into before and after. Something will end — and that ending will open a completely new cycle. At the end of the period you will feel yourself a different person. 
+Relocations, a change of profession, radical changes in lifestyle, the birth of a child as a transition to a new level — all of this is characteristic of the thirteen. Even your style of clothing, circle of contacts, way of thinking — may change completely. 
+In the positive, all changes happen harmoniously — as if everything had been leading to this. Old relationships may be revived, gain a second wind. 
+The main trap is clinging to the old. Whoever holds onto the past — receives destruction without the new. Whoever lets go consciously — receives a qualitatively new life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>13</v>
+      </c>
+      <c r="E646" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Go toward conscious changes — this is the only way to channel this energy into the positive. Declutter your home and gadgets. Close unfinished matters — take inventory and cross off the irrelevant. Arrange a detox for body and mind. Start a renovation or change your image. Quit bad habits — now is the very time. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>14</v>
+      </c>
+      <c r="E647" t="inlineStr">
+        <is>
+          <t>Temperance. Soul and Creativity.** 
+### **Personal forecast** 
+This is a period of maturity and depth. Not speed — but quality. Not storming — but ripening. Everything happens at its own pace, and it’s practically impossible to influence that pace. The task is to trust and observe. 
+The period gives exactly as much as needed — no more and no less. Creativity, self-knowledge, self-development — all of this blossoms. Through art, a potential is revealed that later bears fruit in business and relationships. 
+Moderation in everything — is the key word of the period. Don’t be greedy, don’t rush, don’t chase the excessive. Do everything slowly and well. 
+The main trap is extremes. Excessive consumption — of food, alcohol, entertainment. Or on the contrary — apathy and depression. It’s important to keep yourself in tone and not slide into the minus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D648" t="n">
+        <v>14</v>
+      </c>
+      <c r="E648" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Go to museums, theaters, concerts. Engage in creativity in any form — it is the main resource of the period. Work with water — a conscious shower, baths with salt, bathing in springs. Practice asceticism — a conscious refusal of something in the name of something greater. Work with a psychologist if there are inner torments. Lead a healthy lifestyle. Take photographs — that too is creativity. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D649" t="n">
+        <v>15</v>
+      </c>
+      <c r="E649" t="inlineStr">
+        <is>
+          <t>The Devil. Manifestation and Earthly Pleasures.** 
+### **Personal forecast** 
+One of the most vivid and tempting periods. Money, power, passion, fame — all of it literally falls into your hands. What once required persistent labor — now comes on its own. Life is in full swing, there are many events, the sense that anything is possible. 
+Active manifestation of personality, strong infatuations, passionate romances, admirers — are characteristic of the fifteen. A period of earthly pleasures — delicious food, beautiful clothing, luxurious surroundings. 
+This is precisely where the lesson lies — to hold back from excess. An easy victory and a sense of permissiveness can swallow you up and exalt you above others. And after that — a loud, sobering fall. 
+The main trap is giving in to all the vices. Alcohol, addictions, manipulations, fraud, a dissolute lifestyle. All of it is available — and that is exactly why it’s especially dangerous.</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D650" t="n">
+        <v>15</v>
+      </c>
+      <c r="E650" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Know moderation — that’s the main thing. Practice asceticism and detox — for body, mind, and soul. Work with the shadow sides of the personality. Convert sexual energy into creative energy. Reveal passion through the beauty of life — in every moment. Arrange photoshoots. Having overcome the temptations of this period — you rise to a new level. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>16</v>
+      </c>
+      <c r="E651" t="inlineStr">
+        <is>
+          <t>The Tower. Spiritual Awakening.** 
+### **Personal forecast** 
+This is a period of the destruction of the old for the birth of the new. The Tower doesn’t punish — it frees. Everything that was held up by false foundations — collapses. And this gives the chance to build anew — better, stronger, on a real foundation. 
+A period of building in the literal and figurative sense. Renovation, a change of housing, operations long postponed, radical changes of lifestyle — all of this is activated. Career growth, the resolution of bureaucratic matters, the purchase of real estate — are possible with a conscious living-through. You will feel strength of spirit, insights, heightened awareness. False beliefs leave — a new understanding of life arrives. 
+The main trap is holding onto the old when it is already collapsing. The tighter you cling — the harsher the blow. To accept changes flexibly and consciously — is the only way to pass through the period gently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>16</v>
+      </c>
+      <c r="E652" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Declutter — literally and in everything. Change the space around you — the more global the better. Work with inner aggression. Practice gratitude and deep forgiveness. A detox of body, mind, and soul — is mandatory. Be more careful on the roads. Act for the good of others — this is the main principle of the period. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>17</v>
+      </c>
+      <c r="E653" t="inlineStr">
+        <is>
+          <t>The Star.** 
+### **Personal forecast** 
+This is the time to step onto the stage. To declare yourself. To shine — in your profession, in creativity, in life. Whoever hasn’t yet found themselves — will find it precisely now. Whoever is already on their path — will get vivid results and recognition. 
+Intuition in this period is especially strong — it leads to fateful events and the right people. It’s important to hear the quiet voice of the soul and follow it. 
+Creativity of any kind blossoms — knitting, photography, video, design, music. Social media, public events, going out among people — all of this receives powerful support. A meeting with a very significant person is possible. Romantic, warm relationships — are highly likely. 
+The main trap is a burned-out star. Hiding, slipping into gloom, fearing being in view. Or on the contrary — a star complex and vanity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>17</v>
+      </c>
+      <c r="E654" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Change your image — dare to do what you’ve long dreamed of. Try yourself at what once didn’t work out. Write down what set you alight in childhood — and start doing it. Visualize the desired reality in detail. Control ambitions — in both directions. Shine — that is your task for the period. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D655" t="n">
+        <v>18</v>
+      </c>
+      <c r="E655" t="inlineStr">
+        <is>
+          <t>The Moon. The Hidden and the Lunar.** 
+### **Personal forecast** 
+This is a period of the subconscious, intuition, and illusions. The path isn’t always clearly visible — but it is felt. You will sense that something is happening behind the scenes, that someone is dishonest, that there is something concealed. Logic will resist — but the subconscious knows the truth. 
+The period is full of doubts and ebbs and flows. This is normal. The task is not to fight it but to listen to yourself more attentively than usual. 
+Spiritual work with the subconscious — is a priority. Psychology, astrology, numerology, work with fears and illusions — all of this gives a powerful result precisely now. Creative self-expression blossoms — theater, cinema, fashion, art. 
+Everything you imbue with vivid emotions — materializes. That’s why the choice of thoughts in this period is critically important. Fears come true just as well as dreams. 
+The main trap is negative thoughts, gossip, depressive surroundings, illusions that lead away from reality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>18</v>
+      </c>
+      <c r="E656" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Follow the lunar calendar — in this period the moon influences you especially strongly. Make contact with water — the sea, the pool, baths with salt. Work through fears. Avoid envious and depressive people. Sort your thoughts — throw out the negative ones without regret. Do practices in the second half of the day by candlelight. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>19</v>
+      </c>
+      <c r="E657" t="inlineStr">
+        <is>
+          <t>The Sun. Light and Joy.** 
+### **Personal forecast** 
+One of the best periods in life. You literally shine — and everyone around feels it. Respect, recognition, new useful connections, career heights, material abundance — all of it comes in the period of the nineteen. 
+Much that was hidden — becomes clear. You finally feel the joy of life at full strength. Dream to the maximum and realize yourself fully — that is literally the task of the period. 
+The birth of children, the appearance of new relatives, time spent with children — are characteristic themes. For women a vivid new romance is possible. Marriage — is very favorable. 
+The main trap — in the minus, the sun not only warms but burns. Self-flagellation, fixation on the negative, sharp words that wound loved ones — all of this turns the energy against you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>19</v>
+      </c>
+      <c r="E658" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Do practices in the first half of the day. Early rising and morning activity — are a priority. Declutter from everything outlived. Engage in charity from a pure heart. Work through the fear of poverty — write out negative beliefs about money and replace them. Share knowledge without pride. Be grateful — on a grand scale, for everything. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>20</v>
+      </c>
+      <c r="E659" t="inlineStr">
+        <is>
+          <t>Judgement. Lineage and Clear Knowing.** 
+### **Personal forecast** 
+This is a period of global changes that have long been ripening. You’ve simply finally matured and the time has come. The way things were before — stops being satisfactory. A search for a new path begins. 
+Stepping out onto large horizons — a new level, a relocation, unexpected popularity, going into the public space. If you’ve reached your maximum at work — this energy will push you toward your own venture. Doing something new on the basis of what’s been built up — is the main task of the period. 
+The connection with the lineage becomes especially strong. Positive changes in the family, the birth of children, reunion with relatives, the strengthening of ancestral ties. This is a period when it’s important to work through relationships with both parents. 
+Good news, large money, important decisions that change life for years ahead — are characteristic events of the plus scenario. 
+The main trap is clinging to a past that’s unsatisfactory simply because it’s familiar. Repeating ancestral programs that pull you back.</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>20</v>
+      </c>
+      <c r="E660" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Mend relationships with parents — eliminate grudges and misunderstandings. Compile a family tree — this powerfully boosts the energy of the period. Forgive your mother and father — through a letter, through the practice of constellations, through meditation. Unite the images of both parents behind your back — literally through visualization. Don’t protest against the world — accept, but don’t resign yourself. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>21</v>
+      </c>
+      <c r="E661" t="inlineStr">
+        <is>
+          <t>The World. Expansion and the Universe.** 
+### **Personal forecast** 
+This is a period of completion and expansion at once. Long projects that dragged on for years — finally complete. Long-awaited results arrive. And after this — the whole World opens. In the literal and figurative sense. 
+Relocations, travels, new people, new countries, going onto the international level, large-scale projects — all of this is supported by the energy of the twenty-one. The expansion of consciousness happens on its own — you suddenly understand that what seemed impossible — is easy. Wait, that was allowed all along? 
+A streak of difficulties ends. A time comes to simply live, enjoy, travel, take pleasure in what’s been achieved. 
+The main trap is fears and doubts that prevent action. Debts and loans that limit expansion. Autoaggression and self-flagellation that narrow the world to the size of a problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>21</v>
+      </c>
+      <c r="E662" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Travel — the farther the better. Learn languages. Agree to offers to relocate or try something new. Keep a gratitude journal — at least 10 points a day. Stop warring with yourself — treat yourself like a beloved child. Clear away debts. Visualize your dream travels — through food, languages, the atmosphere of other countries. 
+###</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>22</v>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>The Fool. The Highest Freedom of Spirit.** 
+### **Personal forecast** 
+Everything resets — and a new life begins. A blank page, a new venture, new relationships, a new city, a new image of yourself. The feeling as if you’ve broken free — and everything that held you in a cage before has simply vanished. 
+The period is full of dynamism, adventures, unexpected turns. Travels, new acquaintances, going online, freelancing, unusual activity — all of this is supported by the energy of the twenty-two. Unexpected money and winnings are possible. 
+You will want to embrace everything at once — this is normal. The main thing is not to cling to trifles and daily routine, to live in the flow, to enjoy the here and now. 
+The main trap is recklessness. Reckless risk, addictions, slipping into illusions — alcohol, gambling. A fixation on the material that drags you down like a snowball.</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>FORECAST</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Personal Forecast</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Recommendations</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>22</v>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>for the personal forecast 
+Start something new — this is a mandatory condition of the plus scenario. Release everything that is leaving — without regret. Travel — at least to a neighboring city. Keep a gratitude journal — for what is and for what you want. Awaken the inner child — play, fool around, recall childhood joys. Don’t violate others’ boundaries or the law. Trust the flow. 
+###</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14881,7 +16178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14988,6 +16285,1694 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>The Magician. The Pioneer.** 
+_Only in the personal forecast — in the year of birth and at ages 20, 40, 60 (at 40 and 60 as the second energy)._ 
+This is one of the most powerful periods in a person’s life. Everything you conceive has a chance to take form. Ideas find shape, plans come to life, doors open where before there was a dead end. This is a time of active movement forward. New knowledge, new contacts, new projects. The mind is literally tuned to absorb information — learn, soak it up, grow. Promotions, business launches, creative breakthroughs are all possible. 
+You are seen. You are heard. In this period you are able to inspire others — simply by your presence and your word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>The main trap of this period is overconfidence. A sense of superiority can turn into conflicts and a loss of authority. Watch your documents — mistakes and misunderstandings are possible. Control your thoughts — in this period they materialize with doubled force.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Set goals and write them down. Seek collaboration with professionals. Strengthen the body — especially the spine and the lower part. Practice meditation. Visit places of power. And work on your self-worth — this period manifests exactly as much as you believe in yourself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>The High Priestess. Unity and Harmony.** 
+### _In the personal forecast — in the year of birth, and at ages 10, 20, 40, and 60. In a couple’s forecast it appears extremely rarely._ 
+This is a period of silence and depth. A time when there’s no need to storm and conquer — there’s a need to listen. Listen to yourself, listen to life, trust what is happening. 
+Intuition sharpens to its limit in this period. Information that was long hidden may open to you. Secrets surface, the concealed comes to light. Don’t ask — just observe. The answers will come on their own. 
+This is a soft, spiritual period. A good time for learning, gathering information, developing inner abilities. Relationships with the mother and the women of the lineage come to the foreground — it’s important to harmonize them. Joyful events connected with children are possible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>The main trap is trying to control everything with logic. It doesn’t work here. Also dangerous are intrigues, gossip, participation in others’ games. A third party may appear in the relationship — a woman who brings instability. Watch the information you pass on and receive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Trust your intuition — in this period it is your main instrument. Record important promises in writing. Practice yoga, meditation, pranayama. Create a harmonious space around you. Watch your nutrition — more natural and plant-based. And remember — the world is not divided into black and white.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>When the three appears in the joint forecast — it is one of the best periods for a relationship. The couple literally blossoms. 
+This is a time of closeness, tenderness, sensuality. The relationship is filled with warmth — you want to create coziness, spend time together, spoil one another. The question of children may arise on its own — or the couple will begin to give special attention to the children they already have. Financially the union strengthens — money comes in, joint purchases are possible, investments in real estate, shared creative or business projects. 
+This is a period when the relationship can move to a new level — official registration, shared housing, conversations about family.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>The risk — if one of the partners slips into hysteria, control, or on the contrary into irresponsibility — the energy of the three begins to work against them. Betrayals, jealousy, problems with conception are possible. 
+It’s important that each stays in their own nature — and gives space to the other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Create beauty together — shared dinners, travel, decorating your common space. Talk about desires and dreams. Give time to the body — massage, the pool, shared rest. Support the femininity of the female partner — and the masculinity of the male partner. Don’t take on the role of the other — that is the main condition for passing through this period harmoniously.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>When the four appears in the joint forecast — it is a period when the relationship demands clarity and structure. Chaos and uncertainty don’t work here. The couple must agree — who is responsible for what, how the roles are arranged, where the union is heading. 
+This is a very favorable period for joint financial decisions — opening a business together, major purchases, real estate investments. Everything that requires responsibility and long-term planning — do it precisely now. 
+Stability arrives in the relationship. The couple makes firm decisions about the future — official registration, joint plans, the delineation of responsibility zones. 
+**_A case from my practice._** Anna and Victor came to me — constant quarrels over who pays, who decides, whose word is final. In the couple’s shared forecast stood the four — the energy of power and structure. But I also looked at their personal energies. That year Victor had the seven — the energy of a breakthrough and achievement; he was racing forward, wanting to decide everything himself. And Anna had the three — feminine energy; she wanted warmth, care, to feel like a woman beside a strong man. Hence the conflict: his seven raced ahead like a tank, while the shared four demanded a clear division of roles. I explained: let Victor direct his seven toward 
+finances and big decisions, and Anna in her three create the home and the atmosphere. They did exactly that — and for the first time in years they stopped warring. Each energy fell into its place.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>The main risk of this period is a power struggle within the union. If both pull the blanket toward themselves, both want to be right and in charge — conflicts begin, pressure, and betrayal or rupture become possible. 
+Also dangerous is a tilt in the other direction — when one takes everything on and the other slips into passivity. This breeds resentment and exhaustion. Unfinished conflicts and old grudges especially interfere in this period. Everything that wasn’t spoken — surfaces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Clearly distribute the zones of responsibility — and respect the other’s zone. Don’t interfere where you’re not asked. Set joint goals in writing. Give more time to one another outside of work — cultural leisure, going out together. For the man — show up as a leader in the family. For the woman — inspire rather than compete. It is precisely in this balance that the four unfolds into the positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>When the five appears in the joint forecast — it is a period when the relationship rises to the level of family and lineage. The couple stops being just two people side by side — it becomes a cell with traditions, responsibility, and meaning. 
+This is one of the best times for the official registration of a relationship. The registry office, a wedding, shared housing — all of this receives the support of this energy. An expansion of the family is possible — the birth of a child or heightened attention to children already present. The relationship develops quickly and genuinely. Meeting — marriage — children — it can all spin into motion swiftly and yet correctly. 
+This is also a period when the couple may encounter the influence of parents and lineage. Someone’s traditions, someone’s rules, someone’s opinion about how things should be — all of this comes to the surface. It’s important to build healthy boundaries with both families.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>The main risk is lecturing and attempts to remake the partner. One begins to teach the other how to live correctly — and the relationship turns into a lesson no one asked for. Also dangerous are conflicts around family values — when partners have different ideas about what matters in a family. Problems with the father in one of the partners can strongly affect the relationship in this period. This is worth working through.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Create your own traditions — the ones that belong only to your couple. Don’t let parents and lineage dictate how to build your family. Respect the other’s path — show by example rather than 
+words. Give time to children together. And mend the relationship with the fathers — your own and your partner’s. This will open the energy of the period to its full force.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>6</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>When the six appears in the joint forecast — it is one of the most favorable periods for any relationship. The couple literally bathes in love — tenderness, attention, closeness, passion. This is a time when you want to be together, create beauty, delight in life side by side. Weddings, official registration, romantic travels are possible. Joint creative projects launch easily. Business partnership in this period can also give excellent results. 
+This is a period when the couple makes an important choice — conscious, from love rather than fear. Those who long postponed a decision — finally make it. 
+Communication becomes deeper and warmer. Many heartfelt conversations, shared rest, pleasures — theaters, restaurants, travels, pleasant meetings with friends. 
+**_A case from my practice._** Sofia and Mark had been through a hard year — they drifted apart, almost stopped having heartfelt conversations. In the couple’s shared forecast appeared the six — the energy of love and choice. But the personal energies explained everything. Mark had the eight — a period of balance and rethinking; he had withdrawn into himself, feeling he was investing more. And Sofia had the nine — she craved silence and depth, and had also stepped back. Two people each went into their own energy — while the shared six above them was literally pleading: return to each other. I explained this to them. They started small — dates, heart-to-heart talks, gifts for no reason. The six filled up — and Mark made the proposal he had been postponing for years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>The main risk of this period is betrayals and love triangles. The six tempts — and if there’s unspokenness in the relationship, a lack of attention or closeness, there’s a high chance someone will start looking for it on the side. 
+Also dangerous are situations when one of the partners doesn’t speak of their needs — stays silent, withdraws, accumulates grudges. Openness is needed here. 
+The interference of third parties — friends, relatives — is also characteristic of this period. It’s important not to let others’ opinions influence the choice within the couple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Tell each other about your love — often, specifically, aloud. Give gifts for no reason. Create beauty together — refresh your home space, travel, go to exhibitions and concerts. Speak openly about your desires and needs — don’t expect your partner to guess. Make choices together — from the heart, not from logic. And remember — in this period love literally materializes. Everything you invest in the relationship — returns many times over.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>When the seven appears in the joint forecast — it is a period of movement and shared achievements. A couple that knows how to move as a team — in this period is capable of much. Joint projects, business, relocations, travels — all of this receives powerful support. The relationship is saturated — much activity, events, shared victories. This is not a period of a quiet harbor — it is a period of the road, shoulder to shoulder. And it is precisely this movement that bonds the couple. 
+Relocations and travels together are especially favorable. New places, new impressions, shared adventures — all of this strengthens the union and adds freshness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>7</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>The main risk — both pull in different directions. Each moves toward their own goal and stops noticing the partner. Or one races ahead while the other stands still — and this breeds irritation and distancing. 
+Also dangerous is the aggression that accumulates in this period — if not released into sports and action, it goes into the relationship. Conflicts, quarrels, competition within the couple — all of this is the minus of the period. 
+Love triangles are also possible — especially if one of the partners goes fully into career and forgets about the relationship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>7</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>a common goal — the one you move toward together. Travel — without fail. Do sports together or each on their own — this is critically important for this period. Agree on roles — who is responsible for what in moving forward. Praise each other for victories — even small ones. And don’t forget to stop and simply be together — without goals and plans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>When the eight appears in the joint forecast — it is a period when the relationship undergoes a test of honesty and balance. Everything that was unequal, unfair, left unspoken — comes to the surface. This is not destruction — it is purification. 
+If there was balance in the couple — the period strengthens the union. Karmic rewards arrive for the labor invested in the relationship. Official registration, important joint documents, major deals are possible. 
+This is also a time when the couple rethinks its principles — how we interact, who is responsible for what, whether we treat each other honestly. Such a conversation in this period is especially valuable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>8</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>The main risk is imbalance in the relationship. One invests significantly more than the other — and this becomes unbearable. Or the grudges accumulated over past injustices finally break through. Court and legal questions may touch the couple — division of property, inheritance, documents. It’s important to act honestly and without manipulation. 
+Unfaithfulness in love and divorce — are possible events of the minus scenario. Especially if imbalance accumulated in the couple for a long time and no one dared to speak about it openly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>8</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Talk honestly — who invests how much and what they receive. Not from accusation — from the desire to even out the balance. Keep the promises made to each other — even small ones. Don’t deceive — in anything. Resolve joint legal and financial matters now — the period is favorable. And remember — everything you sow into the relationship in this period will return to you in the next cycle. Sow care and honesty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>9</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>When the nine appears in the joint forecast — it is a period when the couple needs depth, not activity. Not events — but meanings. Not new impressions — but a real conversation about what matters. 
+This is a time when the couple can truly come to know each other. Not at parties and on travels — but in silence, in conversations about life, in a shared search for truth. 
+Spiritual growth together is a very powerful resource of this period. Joint practices, retreats, learning, reading, meditations — all of this brings the couple closer on a level that isn’t reached through ordinary daily life. 
+It’s possible each partner will need their own space and time for solitude. This is normal and doesn’t mean cooling. On the contrary — a partner who has replenished in solitude returns to the relationship alive and real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>9</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>The main risk is the cooling of feelings. The nine can give a sense of detachment — and if the partner doesn’t understand the nature of this period, they perceive the distance as indifference. Grudges and misunderstanding begin. 
+Also dangerous is jealousy out of nowhere — when one withdraws into themselves and the other begins to suspect. Loneliness within the couple and divorce — are possible events of the minus. 
+It’s important to agree that each one’s solitude is not a rejection of the union. It is self-care for the sake of the quality of the relationship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>9</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Give each other space — without grudges and suspicions. Create a tradition of deep conversations — not about daily life, but about life, meanings, dreams. Practice something spiritual together. Spend time in nature — together and each separately. Listen to your partner’s body, not only their words. And remember — silence together is also closeness. Sometimes the deepest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>When the ten appears in the joint forecast — it is one of the most favorable periods for the union. Life tosses the couple gifts — sometimes completely unexpected. Joint travels, financial breakthroughs, happy coincidences — all of this is real. 
+This is a period when the relationship can rise to a completely new level — quickly and naturally. Without effort and struggle. Simply because the time has come. 
+Important events can happen rapidly — a relocation, a new shared opportunity, the unexpected resolution of a long-hanging question. A couple that knows how to trust the flow — gets the maximum from this period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>The main risk — the lightness the period gives can turn into frivolity. One of the partners may get carried away with someone on the side — precisely because everything happens easily and without consequences. This temptation is real. 
+Also if the couple’s karma is negative — the period may bring an unfavorable turn. Losses, forced changes, karmic punishment. 
+Rapid changes can frighten — especially if one of the partners loves stability. It’s important to agree on how you relate to change and to support each other in moments when everything shifts quickly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>10</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Trust the flow together — don’t resist changes if they come. Practice shared gratitude — for the good and for the difficult. Use the opportunities that appear — don’t postpone. Guard the union from light temptations. And remember — in this period life itself leads you where you need to go. The main thing is not to get in its way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>11</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>When the eleven appears in the joint forecast — it is a period of enormous energy within the union. The couple is literally charged — passion, activity, shared accomplishments. This is a time when together you can move mountains. 
+The sexual life is at its peak — vivid, saturated. Pregnancy is possible. Joint projects, business, sports — all of this receives a powerful impulse. 
+The relationship undergoes a test of strength — and it is precisely this test that strengthens the union. A couple that overcomes difficulties together in this period — becomes significantly stronger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>11</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>The main risk — the excess of energy goes into conflicts. Both are charged, both strong, both want it their own way — and a struggle begins. Aggression, pressure, attempts to suppress the partner with one’s strength. 
+Also dangerous is the workaholism of one of the partners — when all the energy goes into career and nothing is left for the relationship. 
+Problems in the sexual life arise precisely when energy is suppressed or goes in the wrong direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>11</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Do sports — together or each on their own. This is critically important for this period. Channel the strength into joint projects rather than against each other. Make sure both rest — fatigue in this period breeds aggression. Speak of passions and desires openly. Support each other in trials — precisely now this is especially important. And remember — the strength within both of you is made for creation, not destruction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>12</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>When the twelve appears in the joint forecast — it is a period when the relationship invites you to look at it from a different angle. Something in the couple turns over — and this can be both a rise to a new level and a serious trial. 
+The period is favorable for spiritual closeness — joint charity, creativity, helping others. A couple that does something meaningful together — strengthens precisely through this. 
+A necessary sacrifice for the sake of future good is possible. Something needs to be released — a habit, a script, a grudge — so that space opens for the new. 
+**_A case from my practice._** Elena and Pavel came to me in a strange state — the union seemed to hang suspended, with no clarity about where it was heading. In the couple’s shared forecast stood the twelve — the energy of pause and a different vision. The personal energies added color. Elena had the nine — she was drawn inward, toward meaning, toward something greater than daily life. And Pavel had the fourteen — the energy of slow ripening; he didn’t want abrupt moves, he needed time. From the outside it looked like stagnation. In reality both were ripening for something new. I suggested they find a shared cause of service — and they began volunteering together at an animal shelter. The twelve unfolded through service, Elena’s nine found meaning, and Pavel’s fourteen let everything mature at the right pace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>The main risk is self-sacrifice. One of the partners begins to sacrifice themselves for the other — and accumulates hidden discontent. Or both get stuck in the victim position and wait for the other to change something. 
+The period may bring a feeling of suspension in the relationship — it’s unclear where the union is heading, there’s no clarity and certainty. This frightens. But it is precisely in this pause that a new understanding is born. 
+Divorce or the relationship’s rise to a fundamentally new level — both options are real depending on how the couple lives through this period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>12</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>for the couple 
+Look at the relationship with fresh eyes — as if seeing it for the first time. What’s good in it that you’ve stopped noticing? What needs to be released for things to get better? Do something meaningful together — charity, a creative project, helping loved ones. Don’t rescue each other without a request — ask whether help is needed. Endure the pause together — don’t destroy what is ripening. And remember — what is leaving now frees space for something better.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>13</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>When the thirteen appears in the joint forecast — it is a period of radical transformation of the relationship. The union changes — deeply, seriously, irreversibly. And this can be both a powerful renewal and an ending. 
+A couple that is ready to change together — rises to a fundamentally new level of closeness. Old patterns are destroyed — and in their place something truly alive is built. This may look like a crisis — but behind it stands a rebirth. 
+Serious joint decisions are possible — relocation, a change of lifestyle, a new joint project, the birth of a child. Everything that once seemed impossible — suddenly becomes real. Old relationships that seemed faded — may gain a second wind precisely in this period. 
+**_A case from my practice_** . Marina and Igor had lived together for twelve years and were on the edge — everything had become gray, mechanical, dead. In the couple’s shared forecast stood the thirteen — the energy of the death of the old and rebirth. And the personal energies led the same way. Igor had the sixteen — the Tower; everything familiar was collapsing inside him. And Marina had the twenty-one — the energy of completing a cycle and stepping into a new world. Three energies of change at once. Many in their place would simply have divorced, deciding love had died. But I explained: the thirteen is not always an end. It is the death of the old for the sake of the new — but only if you go toward the change consciously and together. They took a radical step — sold their apartment, moved to another city, changed everything. The old couple “died” — and in its place a new one was born. A year later they told me they felt as if they had fallen in love all over again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>13</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>The main risk — if one wants to change and the other clings to the old. This breeds powerful tension and can lead to rupture. Divorce in this period — is one of the possible events. Sometimes it’s a plus — leaving what has long stopped working. 
+Also dangerous are chaos, aggression, spontaneous uncontrolled changes. Everything that happens unconsciously — storms hard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>13</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Agree — are you both ready to change? If yes — go toward changes consciously and together. Discuss what needs to be released in the relationship — habits, grudges, outdated roles. Declutter your shared space — literally. Arrange a joint detox — from information noise, from toxic surroundings, from everything that pulls back. And remember — transformation is not the end. It is a rebirth. And what is born afterward — is better than what was.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>14</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>When the fourteen appears in the joint forecast — it is a period of calm and faithful growth of the relationship. Not explosive — but gradual. The union ripens like good wine — slowly but correctly. This is a time when the couple can truly immerse themselves in creativity together. Joint cultural outings, creating something beautiful, travels with spiritual meaning — all of this fills the union with a special depth. 
+Peace in the home — is one of the main blessings of this period. Stability, equilibrium, faithfulness — are characteristic of the fourteen in a couple’s forecast. 
+The relationship becomes more mature. The couple learns not to rush events — but to trust their natural development. And it is precisely in this trust that real closeness is born. 
+What to watch for in the couple 
+The main risk is frayed nerves and delays that begin to irritate. One wants it faster — the other says wait. Conflicts over a difference in pace. 
+Also dangerous are addictions — alcohol, overeating, any extremes — which can disturb the equilibrium in the couple. 
+An unsuccessful partnership and conflicts — are events of the minus scenario when both don’t know how to find balance between desires and reality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>14</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Go to theaters, museums, exhibitions together — feed the soul with beauty. Create something together — let it be even a small joint creative project. Practice joint water procedures — a sauna, spa, bathing. Slow down — don’t rush events in the relationship. Be grateful to each other for what is right now. And maintain moderation in everything — in demands, in expectations, in passions. It is precisely in this moderation — that the depth and longevity of the union lie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>15</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>When the fifteen appears in the joint forecast — it is one of the most sexually charged and passionate periods for the union. The attraction between partners is at its maximum. Energy is bubbling — and it can be directed into the most varied spheres. 
+A financial breakthrough for the couple — is very possible. Large purchases, a successful business, gaining power and influence — all of it is real with a conscious living-through of the period. 
+A couple that knows how to channel this powerful energy into creation — gets the maximum from the period. Vivid joint projects, travels, creativity — all of this fills the union with passion and meaning at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>15</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>The main risk is betrayals and passionate affairs on the side. The fifteen tempts — and if there’s a lack of passion or closeness in the couple, one of the partners may find it outside the union. Also dangerous are addictions that destroy the relationship — alcohol, gambling, destructive habits. Intrigues, manipulations, attempts to control the partner through money or sex — all of these are characteristic risks of the minus scenario. 
+Destructive bonds and self-destruction — are possible if both gave in to the dark side of this period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>15</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Channel the passion into the relationship — literally. Give time to intimate life, beauty, pleasures together. Arrange a joint detox — from everything excessive. Each work with their shadow sides — and speak honestly about temptations without staying silent. Reveal sexuality through creativity — photoshoots together, beautiful evenings, passionate moments. And remember — the power of this 
+period is enormous. The only question is where it’s directed — toward destruction or toward creating something truly vivid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>16</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>When the sixteen appears in the joint forecast — it is a period when the relationship passes through a serious trial. What was unreal — will collapse. What was on a solid foundation — will hold and strengthen. 
+This can be a turning point in the union. A crisis that changes everything. But it is precisely through this crisis that the couple rises to a qualitatively new level — if both are ready to change. A joint relocation, the start of living together, a radical change of lifestyle together — are possible positive events. A couple that builds something new together — gets a powerful impulse from this period. 
+The spiritual awakening that each one experiences — can lead to a deep rethinking of the relationship. This is not frightening. It is necessary. 
+**_A case from my practice_** . Olga and Sergey went through a real storm that year. In the couple’s shared forecast stood the sixteen — the Tower. But I always look at the personal energies of each as well. Sergey had the thirteen in his personal forecast — the energy of collapse and transformation, and indeed: he suddenly lost his job, everything came crashing down. And Olga, in the same period, had the twenty — the energy of lineage and rethinking; she was searching for a new path. Add it up: his personal collapse, her inner search, and the shared Tower of the couple on top. Most would have decided this was the end. But I explained — the Tower destroys only what stood on sand. Sergey, living through his thirteen, didn’t cling to the old but was reborn — he opened his own business. Olga, through her twenty, supported him as a pillar of the lineage. Three energies converged — and instead of collapse they gave a powerful breakthrough. A year and a half later they were stronger and wealthier than ever.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>16</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>The main risk is divorce and rupture if the couple held together out of fear or habit rather than love. The Tower bares the truth — and if the truth is that the union has long been dead, the period will show it. 
+Also dangerous are crises that strike the couple from outside — financial losses, real estate problems, accidents, illnesses. All of this can create enormous pressure on the relationship. Aggression and mutual accusations in a difficult moment — are a characteristic minus of this period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>16</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Don’t fight the changes — accept them together. Declutter as a couple — from grudges, old grievances, outdated agreements. Renew your space — do a renovation or at least rearrange things together. Practice forgiveness — of each other and yourselves. Act for the good of each 
+other and those around you. And remember — everything that collapses in this period collapses because it no longer served you. On the ruins, something better is built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>17</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>When the seventeen appears in the joint forecast — it is a period when the couple comes into the light. Becomes noticeable — both to themselves and to the world around them. This is a time when the union inspires others. A couple that shines together — attracts opportunities, people, events. Joint creativity, public projects, going onto social media together — all of this strengthens both the relationship and self-realization. 
+Romance and beauty within the union — are on the rise. The couple seems to fall in love again. Warm, touching moments, beautiful gestures, attention to one another — all of this is characteristic of the period. 
+Important joint events are possible — marriage, travels, new acquaintances that change the couple’s life.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>17</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>The main risk — one of the partners withdraws into themselves and dims the light. The gloom, insecurity, passivity of one drags the other down too. Or on the contrary — one starts to shine too brightly on their own and the couple loses their shared space. 
+Envy between partners — an unexpected but real risk of this period. If one realizes themselves more brightly — the other may feel themselves in the shadow. 
+Betrayal by friends and loss of faith — are possible events of the minus that can strike the couple from outside.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>17</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Shine together — find what you both can do publicly and with joy. Support each other’s selfrealization — rejoice in your partner’s successes as your own. Refresh your appearance — together or each in their own way. Go to events, go out among people. Visualize your shared desired life — in detail, together. And remember — a star shines brighter when beside it is someone who believes in its light.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>18</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>When the eighteen appears in the joint forecast — it is a period when everything hidden in the relationship comes to the surface. Secrets, unspokenness, illusions that held the couple together — all of it manifests. 
+This can be frightening — but it is precisely this that purifies the union. A couple ready for an honest conversation about what’s happening at the depths — comes out of this period significantly closer and more real. 
+The theme of home, family, children comes to the foreground. The birth of a child, closer contact with parents — are possible events of the period. Joint creativity, art, spiritual practices together — strengthen the union. 
+Romantic acquaintances are possible for those who are searching — the moon attracts beautiful meetings. 
+**_A case from my practice._** Yana and Anton came with the feeling that a wall had risen between them. Yana suspected Anton was hiding something. In the couple’s shared forecast stood the eighteen — the Moon, the energy of the hidden and concealed. The personal energies explained the anxiety. Anton had the eight — he was rethinking his contribution, silently worrying about money and afraid of seeming weak. And Yana had the eighteen in her personal forecast too — her intuition and anxiety were at their peak, she was imagining things that weren’t there. The Moon thickened the fog on both sides. I explained: the only way out is an honest conversation. They talked it all through. There had been no betrayal — only fears and illusions. The eighteen could have destroyed them through suspicion, but through honesty it brought them closer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>18</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>The main risk is deception and illusions. One of the partners may see in the other not who they are — but who they want to see. Or hide something important. The period bares this. Also dangerous are intrigues and the interference of women from outside — friends, mothers, exes — all of them can influence the couple especially actively in this period. 
+Gossip, envy, witchcraft — are characteristic risks of the minus scenario. It sounds mystical — but energetic vulnerability in this period is real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>18</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Be honest with each other — especially about fears and doubts. Don’t accumulate suspicions — speak of them. Practice joint contact with water — a trip to the sea, a sauna together, baths. Follow the lunar cycles and plan important conversations for the waxing moon. Protect your union from others’ opinions and influences. Visualize your shared happy life — with vivid positive emotions. And trust each other’s intuition — in this period it speaks the truth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>19</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>When the nineteen appears in the joint forecast — it is one of the brightest and most joyful periods for the union. The couple literally bathes in warmth and light. Everything that was tense — softens. Everything that was hidden — becomes clear. 
+This is a time of shared achievements and recognition. A couple that shines together — attracts opportunities, money, the right people. Joint projects, charity, going out to mass events together — all of this strengthens the union. 
+The birth of a child — is one of the most characteristic events of the period. Or special attention and time devoted to the children who already exist. Relationships with fathers — your own and your partner’s — come to the foreground. A good time to mend these connections. 
+For the single — vivid romantic acquaintances. For couples — a new round of love and joy. What to watch for in the couple 
+The main risk — one of the partners starts to burn the other. Sharp words, biting criticism, selfflagellation that spills into the relationship — all of this destroys the good that exists. Conflicts with men and problems with fathers — can press on the couple from outside. Childlessness or problems with children — a painful theme in the minus scenario. The loss of status or money in one of the partners — a trial for the union in this period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>19</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Rejoice together — this is the main practice of the period. Go to events, communicate with people, be among the crowd. Devote time to children — your own and others’. Be grateful to each other — every day, specifically and sincerely. Mend relationships with parents — this unblocks the couple’s energy. Share warmth with those around you together — this multiplies it within the union. And remember — in this period your couple can become an example for others. Shine — you have it in you.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>20</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>When the twenty appears in the joint forecast — it is a period when the couple rises to a new level through work with the lineage. The union of two people is always a union of two ancestral systems. And precisely now this is felt especially clearly. 
+A couple that becomes aware of their ancestral programs — and works with them together — gets a powerful breakthrough in this period. Finances, new opportunities, publicity, stepping out onto large horizons — all of this opens through working with the lineage. 
+Often it is precisely in this period that couples decide to have children. Or a merging of families happens — through marriage, through living together, through a family business. 
+Important decisions that change the couple’s life for many years ahead — are made precisely now. Trust this. 
+What to watch for in the couple 
+The main risk is ancestral conflicts that spill into the relationship. Someone’s parents, someone’s relatives, old family grudges — all of this presses on the couple in this period. 
+Repeating negative ancestral programs — when one of the partners behaves like their mother or father in the most destructive manifestations — is a characteristic minus of the twenty. Discord in the family, conflicts with relatives, stagnation due to an unwillingness to change — are events of the minus scenario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>20</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Work with the lineage — each with their own. This is the key practice of the period for a couple. Make peace with parents — both of you. Conduct the practice of uniting the images of mother and father. Study the history of your lineages together — this brings you closer on a surprisingly deep level. Protect your union from others’ ancestral scripts — notice when you start acting not from yourself but from your lineage. And make important decisions now — the period supports everything done consciously and with love for your lineage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>21</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>When the twenty-one appears in the joint forecast — it is a period when the couple literally expands. New horizons open for the union — new countries, new people, new opportunities that previously seemed unattainable. 
+This is a time when long joint plans finally come to life. What you walked toward together for a long time — arrives. The birth of a planned child, laying the foundation of a house, launching a largescale joint project — are characteristic events of the period. 
+Joint travels in this period — are an especially powerful resource. They are not just entertainment — they expand the consciousness of both and open a new dimension in the relationship. The couple’s entry into the public space together — onto the internet, social media, the international level — receives strong support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>21</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>The main risk is fears and distrust of life that keep the couple in a swamp. One wants to expand — the other is afraid. One is ready to relocate — the other clings to the familiar. This creates tension. Debts and financial limitations — can become an obstacle to joint expansion. It’s important not to get into loans that will narrow the couple’s possibilities. 
+The negative thinking of one of the partners — is especially contagious in this period. It literally closes doors that could have opened.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>21</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Travel together — this is the main practice of the period for a couple. Even a small trip to a new place changes something important between two people. Dream big together — and visualize those dreams. Complete everything that has long hung unfinished — and free up space for the new. Agree to the opportunities life offers — even if it’s frightening. Stop warring with each other — the world begins within the union. And remember — in this period the whole world is open before your couple. Literally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Theme</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>22</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>When the twenty-two appears in the joint forecast — it is a period when the couple gets a chance to start everything anew. Not necessarily from scratch — but with a renewed sense of freedom within the union. 
+This is a time when the relationship can rise to a completely unexpected level. A couple that knows how to be light together — gets the maximum from this period. Joint travels, adventures, spontaneous decisions — all of this refreshes and renews the union. 
+The birth of a child, a new joint project, a relocation, going online together — are possible joyful events. An important chance that needs to be caught — appears. Don’t miss it. Freedom within the union — is the key theme of the period. Both must feel that they are not in a cage but in a space where they can breathe. 
+**_A case from my practice._** Karina and Daniel felt stuck — the same walls, the same scenarios, a sense of a cage. In the couple’s shared forecast stood the twenty-two — the energy of reset and a new life. The personal energies amplified it. Daniel had the thirteen — the old in him was dying off, he craved change. And Karina had the twenty-one — the energy of expansion; she longed for the world, movement, space. Everything pointed to one thing: time to start anew. They took the risk — took off on a long journey, then started a joint online project, gave each other the freedom to breathe. The twenty-two reset the old, and the personal energies of each turned it into a new chapter instead of a breakup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>What to watch for in the couple</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>22</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>The main risk is rash decisions made on a wave of freedom. A rupture that happens impulsively and then turns out to be a mistake. Or on the contrary — one of the partners slips into addictions and illusions while the other tries to hold onto reality. 
+Betrayal and the loss of friends — are possible blows from outside that press on the couple. Divorce — in the minus scenario. Especially if one wants freedom and the other holds on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>COMPAT_FORECAST</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Couple Forecast</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Recommendations for the couple</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>22</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Give each other freedom — real freedom. Don’t be jealous of your partner’s life, don’t constrain them. Travel together — this is the main practice of the period. Start something new together — a project, a hobby, an adventure. Be light with each other — play, laugh, fool around. Be grateful for the relationship — both for what’s in it and for what you want. And remember — freedom in a couple is not a threat to the union. It is its air. Where there is air — there is life. 
+## **Conclusion** 
+That’s all. You’ve passed through all twenty-two arcana. You’ve seen how relationships breathe — their high tides and low tides, their rises and trials, their code. And now you know what almost no one knows. 
+You will no longer panic when a difficult period comes. You won’t take a natural dip for the end of love. You won’t leave right before the dawn. You’ll open the forecast, look at the energy of the year — your own, your partner’s, the shared one — and understand what’s happening and why. And having understood — you’ll be able to act. Gently where gentleness is needed. Boldly where the doors are open. 
+This is the meaning of forecasting. It doesn’t take the mystery out of life. It gives you a foundation. It turns fear into understanding, and helplessness into command. You’ve stopped being a passenger. Now you’re at the helm. 
+### **Where to go next** 
+If this book resonated with you — know that it is only a part of the larger world I live in and share. My book “Codes of Compatibility” is a complete guide to relationships through the Matrix of Destiny. About the purpose of your couple — why you met and where you are going together. About karmic tails — the programs that govern your choice of partner. About how each of you truly behaves in a relationship — beneath the masks and the words. 
+A separate guide — “The Betrayal Code.” About what exactly the ancestral system is searching for in a partner, and why betrayal happens. A unique system that isn’t available anywhere in the open. It explains what remained a mystery for years — why people leave, why they cheat, and how to prevent it. 
+### **What’s coming very soon** 
+I am working on a book called “Love Karma” — and it will be the deepest of all my works. If forecasting teaches you to read time, and the Betrayal Code teaches you to understand your partner, then “Love Karma” is about healing. About how to break out of the negative scenarios that repeat from relationship to relationship, from life to life. Why you attract the same type of person again and again. Why you step on the same rake. What karmic knots trail behind you from past incarnations — and how to finally untie them. 
+And a separate major theme of this book — the awakening of sexuality. Liberation from the blocks, shame, and ancestral prohibitions that kept your sensuality locked away for years. A return to yourself — alive, passionate, free. 
+This is a book for those who are tired of going in circles and are ready to truly step out of them. 
+### **Stay close** 
+I share knowledge on social media — breakdowns, insights, living stories from my practice. There I answer questions and show how the Matrix works through real examples. Follow, read, ask questions. I’m here so that you walk this path not blindly — but with light. 
+### **And most importantly** 
+Remember: you are not a passenger in your own life. Not a victim of circumstances, of time, or of others’ decisions. 
+You hold a map. You know the rhythm. You see the energy guiding your union. And now it depends only on you — whether you live your year blindly or consciously. In the minus or in the plus. I believe — you will choose the light. 
+With love and faith in you, 
+Nika Matrix 🖤 
+&lt;!-- Start of picture text --&gt;
+🖤&lt;br&gt;&lt;!-- End of picture text --&gt;</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add Position O interpretations for major arcana 3-9 to data and update parsing tools
</commit_message>
<xml_diff>
--- a/data/interpretations.xlsx
+++ b/data/interpretations.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Documents\matrix\SoulMatrix_latest\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Documents\matrix\extracted 311 22julyupdated\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{08967E3D-63DB-4CA2-BC75-C78A11B1AE81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4732FDF-6626-4860-BE70-180095284078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2739" uniqueCount="607">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2764" uniqueCount="632">
   <si>
     <t>Position</t>
   </si>
@@ -3555,12 +3555,457 @@
 Another difficulty is emotional immaturity. One or both partners may struggle with commitment, avoid responsibility for mistakes or expect love to remain effortless without recognising that healthy relationships require patience, consistency and mutual effort. This can result in repeated cycles of excitement followed by disappointment.
 The relationship becomes stronger when freedom is balanced with responsibility. Keeping a sense of adventure while remaining reliable, communicating honestly and following through on commitments creates trust without losing individuality. The Fool teaches that lasting love does not require giving up freedom. It asks both partners to choose each other willingly each day, creating a relationship that is both exciting and secure.</t>
   </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 3 – The Empress
+### Core Lesson
+The biggest challenge with the Empress at Position O is learning that love is not measured by how much you give, sacrifice or do for other people. Care can easily become control, and support can become overprotection.
+### Common Parent/Child Pattern
+There is often a tendency to become the emotional carer within the family. You may feel responsible for everyone's happiness, believing that if you just give more love, more attention or more support everything will be okay. This can create unhealthy dependence where people stop taking responsibility for themselves.
+### Typical Mistakes
+• Giving far more than you receive.
+• Expecting others to love you in the same way you love them.
+• Becoming overprotective or controlling through care.
+• Taking responsibility for everyone else's happiness.
+• Focusing on practical care while neglecting emotional honesty.
+### Emotional Wound
+Deep down there may be a fear that you are only valued for what you do for other people rather than for simply being yourself. Love can begin to feel conditional upon constant giving.
+### Healing Path
+Healthy love allows people to grow, make mistakes and become independent. Continue being caring and supportive, but allow others to carry their own responsibilities. Learn to receive love as easily as you give it, and remember that genuine connection comes through honest communication as much as practical care.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 4 – The Emperor
+### Core Lesson
+The biggest challenge with the Emperor at Position O is learning that strength does not have to mean control. Structure, discipline and responsibility are valuable, but when taken too far they can create emotional distance and make family relationships feel based on rules rather than love.
+### Common Parent/Child Pattern
+There is often a tendency to become the authority figure within the family. You may believe that keeping everyone organised, protected and disciplined is the best way to show love. This can unintentionally create pressure, leaving little room for emotional expression or individuality.
+### Typical Mistakes
+• Trying to control every situation and every family member.
+• Expecting everyone to live by your standards and rules.
+• Becoming emotionally reserved or uncomfortable expressing affection.
+• Believing strength means never asking for help.
+• Putting responsibility above emotional connection.
+### Emotional Wound
+Deep down there may be a fear that if you relax your standards, everything will fall apart. You may have learned that being dependable is more important than being emotionally available.
+### Healing Path
+True leadership within a family comes from balancing strength with compassion. Create healthy boundaries without becoming controlling. Show love as openly as you show responsibility, allow others to make their own mistakes, and remember that trust grows through understanding as much as discipline.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 5 – The Hierophant
+### Core Lesson
+The biggest challenge with the Hierophant at Position O is learning that wisdom should guide, not control. Strong values, beliefs and traditions can become restrictive when you expect everyone in the family to think, live or behave the same way.
+### Common Parent/Child Pattern
+There is often a tendency to take on the role of teacher, adviser or moral guide within the family. You may genuinely want the best for those you love, but your guidance can become criticism or pressure if you believe your way is the only correct way. Family members may feel judged rather than supported.
+### Typical Mistakes
+• Imposing your beliefs, values or traditions on others.
+• Expecting family members to follow your moral standards.
+• Becoming disappointed when others choose a different path.
+• Refusing to adapt when old family rules no longer serve a purpose.
+• Taking family life too seriously and forgetting warmth and acceptance.
+### Emotional Wound
+Deep down there may be a fear that if people reject your advice, they are rejecting you. This can create frustration when loved ones make choices you would never make yourself.
+### Healing Path
+Share your wisdom without expecting obedience. Respect that every member of the family has their own lessons to learn and their own journey to follow. Encourage rather than preach, remain open to different viewpoints, and remember that acceptance often teaches more than correction.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 6 – The Lovers
+### Core Lesson
+The biggest challenge with the Lovers at Position O is learning that love cannot be controlled, earned or forced. Healthy family relationships are built on acceptance, honesty and freedom, not obligation, guilt or emotional pressure.
+### Common Parent/Child Pattern
+There is often a tendency to place too much importance on approval and acceptance within the family. You may find yourself trying to keep everyone happy, sacrificing your own needs, or believing love has to be earned through your actions. Equally, you may expect those closest to you to make the same choices you would make, believing your way is the best way.
+### Typical Mistakes
+• Sacrificing your own needs to gain love or approval.
+• Feeling responsible for keeping the family happy.
+• Depending too heavily on parental approval.
+• Rejecting your parents' opinions simply to prove your independence.
+• Imposing your own beliefs about love and relationships onto your children.
+• Avoiding difficult choices to keep the peace.
+### Emotional Wound
+Deep down there may be a fear that making your own choices will lead to rejection or disappointment. This can leave you constantly seeking reassurance, approval or validation from those closest to you.
+### Healing Path
+Healthy relationships allow each person the freedom to make their own choices. Love grows through honesty, respect and acceptance, not sacrifice or control. Trust your own heart, respect the different paths of those you love, and allow family relationships to develop naturally without trying to force outcomes.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 7 – The Chariot
+### Core Lesson
+The biggest challenge with the Chariot at Position O is learning that not everyone travels through life at the same speed. Determination and independence are powerful qualities, but they can become controlling when you expect your family to follow your direction or keep up with your pace.
+### Common Parent/Child Pattern
+There is often a strong desire to take charge and keep life moving forward. You may feel responsible for making decisions, solving problems and leading the family. While your intentions are usually positive, loved ones may feel overlooked if their emotions, opinions or personal journey are sacrificed for progress.
+### Typical Mistakes
+• Trying to control the direction of family life.
+• Becoming impatient with those who move more slowly.
+• Prioritising goals and achievements over emotional connection.
+• Believing independence means handling everything alone.
+• Ignoring the emotional needs of family members while focusing on practical results.
+• Expecting children or parents to follow your plans rather than their own path.
+### Emotional Wound
+Deep down there may be a fear that losing control will lead to failure or chaos. This can make it difficult to relax, trust others or allow people the freedom to make their own decisions.
+### Healing Path
+True leadership is about guidance, not control. Learn to balance ambition with empathy, independence with cooperation, and action with emotional understanding. Encourage loved ones to find their own direction while offering support rather than steering every part of their journey.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 8 – Justice
+### Core Lesson
+The biggest challenge with Justice at Position O is learning that fairness does not always mean treating everyone the same. Strong principles, honesty and accountability are valuable, but family relationships also require compassion, understanding and forgiveness.
+### Common Parent/Child Pattern
+There is often a tendency to judge situations through logic rather than emotion. You may expect family members to take responsibility for their actions and believe everyone should be held to the same standards. While this creates integrity, it can also leave loved ones feeling criticised, misunderstood or unable to live up to your expectations.
+### Typical Mistakes
+• Being overly critical or judgmental of parents or children.
+• Expecting perfection or consistently high standards.
+• Finding it difficult to forgive mistakes or let go of the past.
+• Believing rules are more important than emotional understanding.
+• Struggling to show compassion when others fall short.
+• Measuring love through fairness rather than acceptance.
+### Emotional Wound
+Deep down there may be a fear of being treated unfairly or taken advantage of. This can lead you to become defensive, keep score in relationships or expect others to constantly prove themselves.
+### Healing Path
+True fairness combines honesty with compassion. Accept that every family member has different strengths, weaknesses and life lessons. Offer guidance without judgement, forgive imperfections, and remember that unconditional love often heals more than being right ever can.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 9 – The Hermit
+### Core Lesson
+The biggest challenge with the Hermit at Position O is learning that emotional distance is not the same as wisdom. Reflection and independence are valuable strengths, but family relationships also require openness, warmth and genuine connection.
+### Common Parent/Child Pattern
+There is often a tendency to withdraw when emotions become difficult. You may prefer to deal with problems alone, believing that keeping your thoughts to yourself protects both you and your loved ones. While this may feel safer, family members can experience it as rejection, coldness or a lack of interest in their lives.
+### Typical Mistakes
+• Becoming emotionally distant instead of communicating openly.
+• Isolating yourself when family problems arise.
+• Believing you must solve everything alone.
+• Finding it difficult to ask for or accept help.
+• Appearing critical, detached or emotionally unavailable.
+• Expecting others to simply understand how you feel without expressing it.
+### Emotional Wound
+Deep down there may be a fear of being misunderstood, disappointed or emotionally hurt. This can lead you to build walls around yourself, making it difficult for parents, children or other loved ones to truly know what you're feeling.
+### Healing Path
+True wisdom is knowing when to share as well as when to reflect. Allow yourself to be emotionally present, even when conversations feel uncomfortable. Let family members support you, express your feelings honestly, and remember that closeness grows through openness, not silence.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 10 – Wheel of Fortune
+### Core Lesson
+The biggest challenge with the Wheel of Fortune at Position O is learning that family life cannot always be controlled. Change is a natural part of life, and resisting it or expecting stability at all times can create unnecessary stress and disappointment.
+### Common Parent/Child Pattern
+There is often a tendency to rely on circumstances rather than taking consistent responsibility within family relationships. At times you may embrace change and excitement, while at other times you may resist it completely. This inconsistency can leave parents or children feeling uncertain about where they stand with you.
+### Typical Mistakes
+• Avoiding responsibility by believing things will simply work themselves out.
+• Resisting necessary changes within the family.
+• Chasing excitement while neglecting stability.
+• Allowing moods or changing circumstances to influence your commitment to loved ones.
+• Expecting life to improve without making practical changes.
+• Becoming frustrated when family life doesn't go according to plan.
+### Emotional Wound
+Deep down there may be a fear that everything important can change or disappear without warning. This can create anxiety around commitment, making it difficult to trust periods of stability or believe that good times will last.
+### Healing Path
+Accept that change is part of every family's journey. Focus on what you can influence instead of worrying about what you can't control. Build consistency through your actions, remain flexible when life takes unexpected turns, and become a steady source of support regardless of changing circumstances.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 11 – Strength
+### Core Lesson
+The biggest challenge with Strength at Position O is learning that true strength is shown through patience, compassion and emotional balance, not by overpowering others. A strong personality can inspire a family, but it can also become intimidating if your will is placed above everyone else's needs.
+### Common Parent/Child Pattern
+There is often a tendency to take charge during difficult situations, believing you must always be the strong one. You may hide your own vulnerability while expecting others to cope in the same way. Family members can feel they have little space to express weakness or emotion because they believe they need to meet your expectations.
+### Typical Mistakes
+• Trying to dominate situations instead of working together.
+• Suppressing your own emotions to appear strong.
+• Expecting parents or children to be as resilient as you.
+• Becoming impatient with emotional vulnerability or perceived weakness.
+• Using determination to influence or pressure others.
+• Believing asking for help is a sign of weakness.
+### Emotional Wound
+Deep down there may be a fear of losing control or appearing vulnerable. This can make it difficult to trust others with your feelings, leaving you carrying emotional burdens alone while unintentionally pushing loved ones away.
+### Healing Path
+Real strength comes from balancing courage with kindness. Allow yourself to be open about your feelings and give others permission to express theirs without judgement. Support rather than control, encourage rather than pressure, and remember that a family's greatest strength comes from emotional trust, not emotional toughness.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 12 – The Hanged Man
+### Core Lesson
+The biggest challenge with the Hanged Man at Position O is learning that love should not require constant sacrifice. Compassion and patience are beautiful qualities, but repeatedly putting everyone else's needs before your own can lead to resentment, exhaustion and unhealthy family dynamics.
+### Common Parent/Child Pattern
+There is often a tendency to become the one who carries the emotional weight of the family. You may take responsibility for solving everyone else's problems, believing that your own needs can wait. Over time, this can create an imbalance where others become dependent on your support while your own wellbeing is overlooked.
+### Typical Mistakes
+• Constantly sacrificing your own needs for your family.
+• Feeling guilty when putting yourself first.
+• Taking responsibility for problems that belong to others.
+• Staying in unhealthy family situations out of obligation.
+• Believing suffering proves your love or loyalty.
+• Finding it difficult to set healthy emotional boundaries.
+### Emotional Wound
+Deep down there may be a fear that saying "no" will disappoint the people you love or make you appear selfish. This can leave you feeling trapped between caring for others and caring for yourself.
+### Healing Path
+Healthy love includes healthy boundaries. Support your family without carrying burdens that are not yours to bear. Allow others to learn through their own experiences, recognise that your needs matter too, and remember that caring for yourself enables you to care for others from a place of strength rather than sacrifice.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 13 – Death
+### Core Lesson
+The biggest challenge with Death at Position O is learning that endings are not failures. Transformation is a natural part of family life, but resisting change or holding on to the past can prevent both you and your loved ones from growing.
+### Common Parent/Child Pattern
+There is often a tendency to cling to old family roles, painful memories or outdated expectations. You may struggle to let go of past hurts, expecting parents or children to remain the same rather than allowing them to evolve. This can create tension when life naturally moves people in different directions.
+### Typical Mistakes
+• Holding on to past conflicts instead of allowing healing.
+• Resisting necessary changes within the family.
+• Expecting people to remain who they once were.
+• Struggling to forgive or move on from painful experiences.
+• Fearing endings, separation or major life transitions.
+• Trying to control change instead of accepting it.
+### Emotional Wound
+Deep down there may be a fear of loss, abandonment or uncertainty. This can make it difficult to trust life's natural cycles, causing you to hold on to relationships, expectations or emotional pain long after they have served their purpose.
+### Healing Path
+Transformation creates space for new beginnings. Accept that every family relationship changes over time and that growth often requires letting go of old patterns. Forgive where possible, embrace healthy change, and trust that releasing the past allows stronger, healthier relationships to develop in the future.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 14 – Temperance
+### Core Lesson
+The biggest challenge with Temperance at Position O is learning that harmony cannot be created by avoiding conflict. Peace within a family comes through honest communication and healthy balance, not by constantly smoothing things over or putting everyone else's needs before your own.
+### Common Parent/Child Pattern
+There is often a tendency to become the peacemaker within the family. You may naturally try to calm arguments, keep everyone happy and prevent disagreements from escalating. While this creates stability, it can also mean your own feelings are overlooked, or important issues remain unresolved because nobody wants to upset the balance.
+### Typical Mistakes
+• Avoiding difficult conversations to keep the peace.
+• Suppressing your own feelings for the sake of harmony.
+• Becoming the mediator for everyone else's problems.
+• Trying to fix every family disagreement yourself.
+• Ignoring growing resentment until it eventually surfaces.
+• Believing peace is more important than honesty.
+### Emotional Wound
+Deep down there may be a fear that conflict will damage relationships or cause people to drift apart. This can make you overly accommodating, leaving you exhausted while trying to keep everyone else emotionally comfortable.
+### Healing Path
+True harmony is built on honesty as well as kindness. Express your own needs without guilt, allow others to resolve their own disagreements where appropriate, and understand that respectful conflict can strengthen family relationships. Balance caring for others with caring for yourself, and let peace come from authenticity rather than avoidance.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 15 – The Devil
+### Core Lesson
+The biggest challenge with the Devil at Position O is learning that love should never be based on control, fear or emotional dependence. Strong family bonds are healthy, but they become damaging when they are built on manipulation, guilt or the need to keep others close at any cost.
+### Common Parent/Child Pattern
+There is often a tendency to form intense emotional attachments within the family. You may struggle to let go, become overly protective, or find yourself caught in unhealthy patterns of control, jealousy or emotional dependence. Family members may feel obligated rather than free to make their own choices.
+### Typical Mistakes
+• Trying to control parents or children through guilt or emotional pressure.
+• Becoming overly attached or unable to let go.
+• Creating unhealthy dependence instead of encouraging independence.
+• Allowing fear, jealousy or possessiveness to influence family relationships.
+• Repeating toxic family patterns because they feel familiar.
+• Confusing control with love and protection.
+### Emotional Wound
+Deep down there may be a fear of abandonment, rejection or losing the people you love. This fear can lead you to hold on too tightly, making it difficult to trust that healthy relationships can survive without constant control or reassurance.
+### Healing Path
+Love grows strongest when people are free to choose each other. Release the need to control outcomes or hold family members too tightly. Encourage independence, break unhealthy emotional patterns, and build relationships based on trust, honesty and mutual respect rather than fear or obligation.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 16 – The Tower
+### Core Lesson
+The biggest challenge with the Tower at Position O is learning that honesty and change do not have to destroy relationships. Sudden truths, conflict or major life changes can become opportunities for growth when they are handled with understanding rather than anger or blame.
+### Common Parent/Child Pattern
+There is often a tendency for family relationships to go through periods of upheaval or dramatic change. You may speak with brutal honesty, react impulsively during conflict, or feel the need to completely break away from old family patterns. While transformation is necessary, it can sometimes happen in ways that leave emotional damage behind if handled without care.
+### Typical Mistakes
+• Reacting impulsively during family disagreements.
+• Using harsh words that are difficult to take back.
+• Believing drastic action is the only way to solve problems.
+• Cutting people off instead of working through conflict.
+• Resisting change until situations reach breaking point.
+• Creating unnecessary disruption through impatience or frustration.
+### Emotional Wound
+Deep down there may be a fear that stability is temporary and that relationships can collapse without warning. This can leave you expecting conflict, preparing for the worst, or unconsciously creating upheaval before life does it for you.
+### Healing Path
+Real transformation doesn't always require destruction. Learn to address problems before they become crises, communicate honestly without becoming hurtful, and allow change to happen gradually where possible. Strong family relationships are built by repairing cracks before the whole foundation begins to shake.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 17 – The Star
+### Core Lesson
+The biggest challenge with the Star at Position O is learning that hope should be balanced with action. Inspiration, optimism and faith can strengthen a family, but unrealistic expectations or avoiding reality can leave important issues unresolved.
+### Common Parent/Child Pattern
+There is often a natural desire to encourage, inspire and see the best in your family. You may believe that everything will work out in the end, sometimes overlooking practical problems or avoiding difficult conversations. At other times, you may place parents or children on a pedestal, expecting more from them than they are able to give.
+### Typical Mistakes
+• Expecting family relationships to be perfect.
+• Avoiding difficult realities in favour of wishful thinking.
+• Placing parents or children on a pedestal.
+• Becoming disappointed when people fail to meet your ideals.
+• Offering encouragement without addressing practical problems.
+• Losing motivation when reality doesn't match your expectations.
+### Emotional Wound
+Deep down there may be a fear that if you stop believing everything will work out, hope will disappear altogether. This can make it difficult to face painful truths or accept that even loving families experience challenges and imperfections.
+### Healing Path
+Hope becomes most powerful when it is supported by honesty and action. Continue inspiring those you love, but accept them as they truly are rather than who you wish them to be. Balance optimism with realistic expectations, address problems openly, and allow authentic relationships to grow from acceptance rather than perfection.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 18 – The Moon
+### Core Lesson
+The biggest challenge with the Moon at Position O is learning to separate fear from reality. Sensitivity and intuition are valuable gifts, but when they become clouded by worry, suspicion or unspoken emotions, family relationships can become confusing and emotionally draining.
+### Common Parent/Child Pattern
+There is often a tendency for misunderstandings, hidden feelings or unspoken expectations to develop within the family. You may avoid discussing difficult emotions, assume you know what others are thinking, or allow fear and uncertainty to shape your reactions. This can create distance even when everyone genuinely cares about one another.
+### Typical Mistakes
+• Avoiding honest conversations about difficult emotions.
+• Assuming the worst instead of asking for the truth.
+• Allowing fear or anxiety to influence family decisions.
+• Keeping secrets or hiding your true feelings.
+• Becoming emotionally unpredictable or difficult to read.
+• Letting misunderstandings grow instead of resolving them.
+### Emotional Wound
+Deep down there may be a fear of betrayal, rejection or being emotionally hurt. This can make it difficult to fully trust parents, children or those closest to you, causing you to withdraw or become overly cautious even when love is present.
+### Healing Path
+Clarity begins with honesty. Share your feelings openly instead of expecting others to guess what you need. Question fearful assumptions before accepting them as facts, trust your intuition without letting fear control it, and create family relationships built on openness, understanding and emotional safety.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 19 – The Sun
+### Core Lesson
+The biggest challenge with the Sun at Position O is learning that confidence should uplift others, not overshadow them. Warmth, generosity and positivity are wonderful qualities, but they can become overwhelming when your need to lead, protect or be recognised leaves little room for others to shine.
+### Common Parent/Child Pattern
+There is often a strong desire to create a happy, successful and close-knit family. You may naturally take on the role of encourager, provider or leader, wanting the very best for those you love. However, there can also be a tendency to expect appreciation, admiration or loyalty in return, leaving family members feeling pressured to meet your expectations rather than simply be themselves.
+### Typical Mistakes
+• Expecting recognition for everything you do for your family.
+• Wanting family members to live up to your ideals or ambitions.
+• Becoming overprotective or overly involved in their lives.
+• Struggling to accept criticism or different opinions.
+• Believing you always know what is best for everyone.
+• Accidentally overshadowing the individuality of parents or children.
+### Emotional Wound
+Deep down there may be a fear of not being valued or appreciated for everything you give. This can lead to disappointment when your love, effort or support isn't recognised in the way you hoped.
+### Healing Path
+True warmth allows everyone to shine. Continue encouraging and supporting your family, but celebrate their individuality rather than shaping them in your image. Give without expecting praise, listen as much as you lead, and remember that the strongest family relationships are built on mutual respect rather than admiration.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 20 – Judgement
+### Core Lesson
+The biggest challenge with Judgement at Position O is learning that healing comes through acceptance, not blame. Family relationships often carry deep ancestral patterns, but repeatedly revisiting the past or judging yourself and others prevents true growth and reconciliation.
+### Common Parent/Child Pattern
+There is often a strong awareness of family history and inherited behaviours. You may feel responsible for healing generational wounds or correcting the mistakes of previous generations. While this can become a powerful gift, it may also lead to carrying burdens that were never yours or becoming overly critical of parents, children or yourself.
+### Typical Mistakes
+• Holding on to resentment about past family experiences.
+• Blaming parents or previous generations for present difficulties.
+• Feeling responsible for fixing everyone else's emotional wounds.
+• Judging yourself too harshly for family mistakes.
+• Repeating generational patterns without recognising them.
+• Becoming so focused on the past that you struggle to enjoy the present.
+### Emotional Wound
+Deep down there may be a fear that the past will continue to define your future. You may worry that family history, inherited behaviours or old emotional wounds can never truly be healed, leaving you feeling responsible for carrying the weight of generations.
+### Healing Path
+Healing begins when you acknowledge the past without allowing it to control your future. Forgive where possible, release burdens that do not belong to you, and recognise that every generation has the opportunity to create a new story. By changing your own patterns, you give both your ancestors and your descendants the gift of transformation.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 21 – The World
+### Core Lesson
+The biggest challenge with the World at Position O is learning that supporting others doesn't mean carrying the whole world on your shoulders. Unity, wisdom and a broad outlook are wonderful gifts, but trying to keep everyone together or solve everyone's problems can leave you emotionally exhausted.
+### Common Parent/Child Pattern
+There is often a natural desire to create a strong, united family where everyone feels connected. You may become the organiser, the peacekeeper or the person everyone turns to for advice. While this creates stability, it can also lead to taking on responsibilities that belong to other family members, making it difficult for them to grow independently.
+### Typical Mistakes
+• Taking responsibility for keeping the whole family together.
+• Feeling personally responsible for everyone else's happiness.
+• Becoming over-involved in relatives' lives or decisions.
+• Finding it difficult to let family members make their own mistakes.
+• Carrying emotional burdens that don't belong to you.
+• Neglecting your own needs while supporting everyone else.
+### Emotional Wound
+Deep down there may be a fear that if you stop holding everything together, the family will fall apart. This can leave you constantly carrying responsibility, even when others are capable of managing their own lives.
+### Healing Path
+Healthy families thrive when responsibility is shared. Continue bringing people together, but allow each person to carry their own lessons and make their own choices. Trust that love does not depend on you fixing every problem, and remember that your role is to support, not to carry the weight of the entire family.</t>
+  </si>
+  <si>
+    <t>## POSITION O – POSSIBLE MISTAKES IN RELATIONSHIPS WITH PARENTS &amp; CHILDREN
+### Arcana 22 – The Fool
+### Core Lesson
+The biggest challenge with the Fool at Position O is learning that freedom and responsibility can exist together. A playful, spontaneous spirit brings joy to family life, but avoiding commitment or refusing to grow up can create instability for those who rely on you.
+### Common Parent/Child Pattern
+There is often a strong desire to live life on your own terms, encouraging independence and freedom within the family. While this can create open-minded and adventurous relationships, there may also be a tendency to avoid difficult responsibilities, make impulsive decisions or dismiss serious family matters too lightly. Parents or children may feel uncertain because they never quite know what to expect.
+### Typical Mistakes
+• Avoiding responsibility or difficult family conversations.
+• Acting impulsively without considering the consequences for others.
+• Resisting commitment or long-term responsibilities.
+• Escaping problems instead of dealing with them directly.
+• Encouraging freedom without providing enough stability or guidance.
+• Treating serious family issues too casually.
+### Emotional Wound
+Deep down there may be a fear that commitment will take away your freedom or that responsibility will stop you living life on your own terms. This can make it difficult to fully settle into family roles or trust that stability doesn't have to mean losing yourself.
+### Healing Path
+Freedom becomes far more meaningful when it is balanced with responsibility. Continue bringing joy, curiosity and fresh perspectives to your family, but show up consistently for the people who depend on you. Honour your independence while creating a safe, reliable foundation where love and trust can flourish.</t>
+  </si>
+  <si>
+    <t>Program</t>
+  </si>
+  <si>
+    <t>Violation Of Hierachy</t>
+  </si>
+  <si>
+    <t>05-08-21</t>
+  </si>
+  <si>
+    <t>L2-L1-L</t>
+  </si>
+  <si>
+    <t># Program 5–8–21 – Violation of Hierarchy
+## The Main Lesson
+This programme is all about respecting the natural order of things, knowing your place within the family or a group, and allowing everyone else to stand in theirs.
+---
+# In the Shadow
+## "I'll Sort It Out"
+This programme often shows up when people start taking on roles that were never theirs to carry.
+This can happen in:
+- A child becoming the emotional parent to their mum or dad.
+- A wife trying to control or parent her husband.
+- Someone at work constantly undermining the boss and trying to take charge.
+Most people aren't doing it to be difficult. They're usually trying to help, protect or fix things.
+The problem is that the natural flow gets turned upside down.
+Children become parents.
+Partners become controllers.
+Support turns into control.
+Over time this can lead to:
+- Feeling emotionally or physically exhausted.
+- Carrying responsibilities that were never yours.
+- Family tension and constant conflict.
+- Power struggles in relationships or at work.
+- In some cases, energetic blocks around fertility or creating new life.
+When everyone starts standing in the wrong place, the whole system becomes unstable.
+---
+# In Balance
+## "Everyone Has Their Rightful Place"
+When this programme is healed, everything begins to flow much more naturally.
+You understand that every person has their own role, lessons and responsibilities.
+Instead of taking over, you allow others to grow through their own experiences while still offering support when it's genuinely needed.
+You realise that:
+- Helping doesn't mean controlling.
+- Leading doesn't mean dominating.
+- Supporting someone doesn't mean rescuing them.
+Respecting the natural order creates harmony in families, relationships, friendships and the workplace.
+---
+# Positive Traits
+- Strong respect for healthy boundaries.
+- Everyone is encouraged to take responsibility for themselves.
+- Able to accept help without guilt or shame.
+- Supports others without taking over their lives.
+- Creates balance and harmony within families and teams.
+---
+# Shadow Traits
+- Parent and child roles become reversed.
+- Trying to control partners, parents or other family members.
+- Caring becomes controlling.
+- Constantly challenging authority or believing you know better than everyone else.
+---
+# Life Lesson
+Respect the natural order.
+Allow people to stand in their own place, even when it's difficult to watch.
+Support people without carrying their responsibilities.
+Your role isn't to take over someone else's path.
+Your lesson is to honour the structure, trust the process and allow life to flow as it should.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3574,6 +4019,12 @@
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3604,7 +4055,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3627,6 +4078,11 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3822,7 +4278,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E664"/>
+  <dimension ref="A1:E665"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -10570,7 +11026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="400" spans="1:5">
+    <row r="400" spans="1:5" ht="406">
       <c r="A400" t="s">
         <v>345</v>
       </c>
@@ -10583,8 +11039,11 @@
       <c r="D400">
         <v>3</v>
       </c>
-    </row>
-    <row r="401" spans="1:4">
+      <c r="E400" s="3" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="401" spans="1:5" ht="409.5">
       <c r="A401" t="s">
         <v>345</v>
       </c>
@@ -10597,8 +11056,11 @@
       <c r="D401">
         <v>4</v>
       </c>
-    </row>
-    <row r="402" spans="1:4">
+      <c r="E401" s="3" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="402" spans="1:5" ht="409.5">
       <c r="A402" t="s">
         <v>345</v>
       </c>
@@ -10611,8 +11073,11 @@
       <c r="D402">
         <v>5</v>
       </c>
-    </row>
-    <row r="403" spans="1:4">
+      <c r="E402" s="3" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="403" spans="1:5" ht="409.5">
       <c r="A403" t="s">
         <v>345</v>
       </c>
@@ -10625,8 +11090,11 @@
       <c r="D403">
         <v>6</v>
       </c>
-    </row>
-    <row r="404" spans="1:4">
+      <c r="E403" s="3" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="404" spans="1:5" ht="409.5">
       <c r="A404" t="s">
         <v>345</v>
       </c>
@@ -10639,8 +11107,11 @@
       <c r="D404">
         <v>7</v>
       </c>
-    </row>
-    <row r="405" spans="1:4">
+      <c r="E404" s="3" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="405" spans="1:5" ht="409.5">
       <c r="A405" t="s">
         <v>345</v>
       </c>
@@ -10653,8 +11124,11 @@
       <c r="D405">
         <v>8</v>
       </c>
-    </row>
-    <row r="406" spans="1:4">
+      <c r="E405" s="3" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="406" spans="1:5" ht="409.5">
       <c r="A406" t="s">
         <v>345</v>
       </c>
@@ -10667,8 +11141,11 @@
       <c r="D406">
         <v>9</v>
       </c>
-    </row>
-    <row r="407" spans="1:4">
+      <c r="E406" s="3" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="407" spans="1:5" ht="409.5">
       <c r="A407" t="s">
         <v>345</v>
       </c>
@@ -10681,8 +11158,11 @@
       <c r="D407">
         <v>10</v>
       </c>
-    </row>
-    <row r="408" spans="1:4">
+      <c r="E407" s="3" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="408" spans="1:5" ht="409.5">
       <c r="A408" t="s">
         <v>345</v>
       </c>
@@ -10695,8 +11175,11 @@
       <c r="D408">
         <v>11</v>
       </c>
-    </row>
-    <row r="409" spans="1:4">
+      <c r="E408" s="3" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="409" spans="1:5" ht="409.5">
       <c r="A409" t="s">
         <v>345</v>
       </c>
@@ -10709,8 +11192,11 @@
       <c r="D409">
         <v>12</v>
       </c>
-    </row>
-    <row r="410" spans="1:4">
+      <c r="E409" s="3" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="410" spans="1:5" ht="409.5">
       <c r="A410" t="s">
         <v>345</v>
       </c>
@@ -10723,8 +11209,11 @@
       <c r="D410">
         <v>13</v>
       </c>
-    </row>
-    <row r="411" spans="1:4">
+      <c r="E410" s="3" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="411" spans="1:5" ht="409.5">
       <c r="A411" t="s">
         <v>345</v>
       </c>
@@ -10737,8 +11226,11 @@
       <c r="D411">
         <v>14</v>
       </c>
-    </row>
-    <row r="412" spans="1:4">
+      <c r="E411" s="3" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="412" spans="1:5" ht="409.5">
       <c r="A412" t="s">
         <v>345</v>
       </c>
@@ -10751,8 +11243,11 @@
       <c r="D412">
         <v>15</v>
       </c>
-    </row>
-    <row r="413" spans="1:4">
+      <c r="E412" s="3" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="413" spans="1:5" ht="409.5">
       <c r="A413" t="s">
         <v>345</v>
       </c>
@@ -10765,8 +11260,11 @@
       <c r="D413">
         <v>16</v>
       </c>
-    </row>
-    <row r="414" spans="1:4">
+      <c r="E413" s="3" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="414" spans="1:5" ht="409.5">
       <c r="A414" t="s">
         <v>345</v>
       </c>
@@ -10779,8 +11277,11 @@
       <c r="D414">
         <v>17</v>
       </c>
-    </row>
-    <row r="415" spans="1:4">
+      <c r="E414" s="3" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="415" spans="1:5" ht="409.5">
       <c r="A415" t="s">
         <v>345</v>
       </c>
@@ -10793,8 +11294,11 @@
       <c r="D415">
         <v>18</v>
       </c>
-    </row>
-    <row r="416" spans="1:4">
+      <c r="E415" s="3" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="416" spans="1:5" ht="409.5">
       <c r="A416" t="s">
         <v>345</v>
       </c>
@@ -10807,8 +11311,11 @@
       <c r="D416">
         <v>19</v>
       </c>
-    </row>
-    <row r="417" spans="1:4">
+      <c r="E416" s="3" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="417" spans="1:5" ht="409.5">
       <c r="A417" t="s">
         <v>345</v>
       </c>
@@ -10821,8 +11328,11 @@
       <c r="D417">
         <v>20</v>
       </c>
-    </row>
-    <row r="418" spans="1:4">
+      <c r="E417" s="3" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="418" spans="1:5" ht="409.5">
       <c r="A418" t="s">
         <v>345</v>
       </c>
@@ -10835,8 +11345,11 @@
       <c r="D418">
         <v>21</v>
       </c>
-    </row>
-    <row r="419" spans="1:4">
+      <c r="E418" s="3" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="419" spans="1:5" ht="409.5">
       <c r="A419" t="s">
         <v>345</v>
       </c>
@@ -10849,8 +11362,11 @@
       <c r="D419">
         <v>22</v>
       </c>
-    </row>
-    <row r="420" spans="1:4">
+      <c r="E419" s="3" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="420" spans="1:5">
       <c r="A420" t="s">
         <v>347</v>
       </c>
@@ -10864,7 +11380,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="421" spans="1:4">
+    <row r="421" spans="1:5">
       <c r="A421" t="s">
         <v>347</v>
       </c>
@@ -10878,7 +11394,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="422" spans="1:4">
+    <row r="422" spans="1:5">
       <c r="A422" t="s">
         <v>347</v>
       </c>
@@ -10892,7 +11408,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="423" spans="1:4">
+    <row r="423" spans="1:5">
       <c r="A423" t="s">
         <v>347</v>
       </c>
@@ -10906,7 +11422,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="424" spans="1:4">
+    <row r="424" spans="1:5">
       <c r="A424" t="s">
         <v>347</v>
       </c>
@@ -10920,7 +11436,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="425" spans="1:4">
+    <row r="425" spans="1:5">
       <c r="A425" t="s">
         <v>347</v>
       </c>
@@ -10934,7 +11450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="426" spans="1:4">
+    <row r="426" spans="1:5">
       <c r="A426" t="s">
         <v>347</v>
       </c>
@@ -10948,7 +11464,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="427" spans="1:4">
+    <row r="427" spans="1:5">
       <c r="A427" t="s">
         <v>347</v>
       </c>
@@ -10962,7 +11478,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="428" spans="1:4">
+    <row r="428" spans="1:5">
       <c r="A428" t="s">
         <v>347</v>
       </c>
@@ -10976,7 +11492,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="429" spans="1:4">
+    <row r="429" spans="1:5">
       <c r="A429" t="s">
         <v>347</v>
       </c>
@@ -10990,7 +11506,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="430" spans="1:4">
+    <row r="430" spans="1:5">
       <c r="A430" t="s">
         <v>347</v>
       </c>
@@ -11004,7 +11520,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="431" spans="1:4">
+    <row r="431" spans="1:5">
       <c r="A431" t="s">
         <v>347</v>
       </c>
@@ -11018,7 +11534,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="432" spans="1:4">
+    <row r="432" spans="1:5">
       <c r="A432" t="s">
         <v>347</v>
       </c>
@@ -14551,6 +15067,23 @@
       </c>
       <c r="E664" t="s">
         <v>416</v>
+      </c>
+    </row>
+    <row r="665" spans="1:5" ht="409.5">
+      <c r="A665" s="10" t="s">
+        <v>630</v>
+      </c>
+      <c r="B665" t="s">
+        <v>627</v>
+      </c>
+      <c r="C665" t="s">
+        <v>628</v>
+      </c>
+      <c r="D665" s="9" t="s">
+        <v>629</v>
+      </c>
+      <c r="E665" s="11" t="s">
+        <v>631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>